<commit_message>
Major Architecture Upgrade: Direct Excel loading, strict business lead-day rules, intelligent guest scaling, and normalized extended stay parsing into 24H Night
</commit_message>
<xml_diff>
--- a/backend/data/Farm_Booking_Data.xlsx
+++ b/backend/data/Farm_Booking_Data.xlsx
@@ -481,7 +481,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-08-05</t>
+          <t>2024-08-06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-08-08</t>
+          <t>2024-08-09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -573,7 +573,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-08-17</t>
+          <t>2024-08-18</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -596,10 +596,10 @@
         <v>7</v>
       </c>
       <c r="G4" t="n">
-        <v>11750</v>
+        <v>9370</v>
       </c>
       <c r="H4" t="n">
-        <v>11040</v>
+        <v>8660</v>
       </c>
       <c r="I4" t="n">
         <v>23.3</v>
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-08-18</t>
+          <t>2024-08-19</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -642,10 +642,10 @@
         <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="H5" t="n">
-        <v>9600</v>
+        <v>7600</v>
       </c>
       <c r="I5" t="n">
         <v>23.9</v>
@@ -665,7 +665,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-08-18</t>
+          <t>2024-08-19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -711,7 +711,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-08-24</t>
+          <t>2024-08-25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -734,10 +734,10 @@
         <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>20650</v>
+        <v>16650</v>
       </c>
       <c r="H7" t="n">
-        <v>20650</v>
+        <v>16650</v>
       </c>
       <c r="I7" t="n">
         <v>26.5</v>
@@ -757,7 +757,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-08-24</t>
+          <t>2024-08-25</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -780,10 +780,10 @@
         <v>4</v>
       </c>
       <c r="G8" t="n">
-        <v>12290</v>
+        <v>9920</v>
       </c>
       <c r="H8" t="n">
-        <v>12990</v>
+        <v>10620</v>
       </c>
       <c r="I8" t="n">
         <v>22.2</v>
@@ -803,7 +803,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-08-25</t>
+          <t>2024-08-26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -826,10 +826,10 @@
         <v>8</v>
       </c>
       <c r="G9" t="n">
-        <v>9530</v>
+        <v>7530</v>
       </c>
       <c r="H9" t="n">
-        <v>9570</v>
+        <v>7570</v>
       </c>
       <c r="I9" t="n">
         <v>24.1</v>
@@ -849,7 +849,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-08-31</t>
+          <t>2024-09-01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -872,10 +872,10 @@
         <v>27</v>
       </c>
       <c r="G10" t="n">
-        <v>7730</v>
+        <v>9730</v>
       </c>
       <c r="H10" t="n">
-        <v>7540</v>
+        <v>9540</v>
       </c>
       <c r="I10" t="n">
         <v>23.3</v>
@@ -895,7 +895,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-09-05</t>
+          <t>2024-09-06</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -941,7 +941,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-09-07</t>
+          <t>2024-09-08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -964,10 +964,10 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>15740</v>
+        <v>19360</v>
       </c>
       <c r="H12" t="n">
-        <v>15890</v>
+        <v>19510</v>
       </c>
       <c r="I12" t="n">
         <v>27.7</v>
@@ -987,7 +987,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-09-13</t>
+          <t>2024-09-14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1033,7 +1033,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-09-13</t>
+          <t>2024-09-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1079,7 +1079,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2024-09-20</t>
+          <t>2024-09-21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1102,10 +1102,10 @@
         <v>8</v>
       </c>
       <c r="G15" t="n">
-        <v>9080</v>
+        <v>11450</v>
       </c>
       <c r="H15" t="n">
-        <v>9250</v>
+        <v>11620</v>
       </c>
       <c r="I15" t="n">
         <v>23.9</v>
@@ -1125,7 +1125,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2024-09-25</t>
+          <t>2024-09-26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1171,7 +1171,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2024-10-01</t>
+          <t>2024-10-02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2024-10-05</t>
+          <t>2024-10-06</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1240,10 +1240,10 @@
         <v>20</v>
       </c>
       <c r="G18" t="n">
-        <v>20640</v>
+        <v>16640</v>
       </c>
       <c r="H18" t="n">
-        <v>21080</v>
+        <v>17080</v>
       </c>
       <c r="I18" t="n">
         <v>20.1</v>
@@ -1263,7 +1263,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2024-10-07</t>
+          <t>2024-10-08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1309,7 +1309,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2024-10-14</t>
+          <t>2024-10-15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1355,7 +1355,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2024-10-23</t>
+          <t>2024-10-24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1401,7 +1401,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2024-10-30</t>
+          <t>2024-10-31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1447,7 +1447,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2024-11-03</t>
+          <t>2024-11-04</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1470,10 +1470,10 @@
         <v>34</v>
       </c>
       <c r="G23" t="n">
-        <v>8170</v>
+        <v>6170</v>
       </c>
       <c r="H23" t="n">
-        <v>7520</v>
+        <v>5520</v>
       </c>
       <c r="I23" t="n">
         <v>18</v>
@@ -1493,7 +1493,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2024-11-07</t>
+          <t>2024-11-08</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1539,7 +1539,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2024-11-10</t>
+          <t>2024-11-11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1585,7 +1585,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2024-11-11</t>
+          <t>2024-11-12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2024-11-14</t>
+          <t>2024-11-15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1677,7 +1677,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2024-11-17</t>
+          <t>2024-11-18</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1723,7 +1723,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2024-11-18</t>
+          <t>2024-11-19</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1769,7 +1769,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2024-12-03</t>
+          <t>2024-12-04</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1815,7 +1815,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>2024-12-11</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1861,7 +1861,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-13</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2024-12-13</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2024-12-16</t>
+          <t>2024-12-17</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2024-12-20</t>
+          <t>2024-12-21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2022,10 +2022,10 @@
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>13840</v>
+        <v>16210</v>
       </c>
       <c r="H35" t="n">
-        <v>14330</v>
+        <v>16700</v>
       </c>
       <c r="I35" t="n">
         <v>20.4</v>
@@ -2045,7 +2045,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2025-01-07</t>
+          <t>2025-01-08</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2025-01-11</t>
+          <t>2025-01-12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2114,10 +2114,10 @@
         <v>14</v>
       </c>
       <c r="G37" t="n">
-        <v>22150</v>
+        <v>18150</v>
       </c>
       <c r="H37" t="n">
-        <v>21810</v>
+        <v>17810</v>
       </c>
       <c r="I37" t="n">
         <v>22.5</v>
@@ -2137,7 +2137,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2025-01-12</t>
+          <t>2025-01-13</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2160,10 +2160,10 @@
         <v>12</v>
       </c>
       <c r="G38" t="n">
-        <v>15370</v>
+        <v>11750</v>
       </c>
       <c r="H38" t="n">
-        <v>15950</v>
+        <v>12330</v>
       </c>
       <c r="I38" t="n">
         <v>20.7</v>
@@ -2183,7 +2183,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2025-01-17</t>
+          <t>2025-01-18</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>2025-02-08</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2275,7 +2275,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2025-02-09</t>
+          <t>2025-02-10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2298,10 +2298,10 @@
         <v>5</v>
       </c>
       <c r="G41" t="n">
-        <v>9430</v>
+        <v>7430</v>
       </c>
       <c r="H41" t="n">
-        <v>9470</v>
+        <v>7470</v>
       </c>
       <c r="I41" t="n">
         <v>23.2</v>
@@ -2321,7 +2321,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>2025-02-12</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2367,7 +2367,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2025-02-20</t>
+          <t>2025-02-21</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2413,7 +2413,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>2025-02-22</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2459,7 +2459,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2025-02-25</t>
+          <t>2025-02-26</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2505,7 +2505,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2025-02-26</t>
+          <t>2025-02-27</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2551,7 +2551,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2025-03-06</t>
+          <t>2025-03-07</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2025-03-08</t>
+          <t>2025-03-09</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2620,10 +2620,10 @@
         <v>30</v>
       </c>
       <c r="G48" t="n">
-        <v>8160</v>
+        <v>10160</v>
       </c>
       <c r="H48" t="n">
-        <v>7480</v>
+        <v>9480</v>
       </c>
       <c r="I48" t="n">
         <v>35.1</v>
@@ -2643,7 +2643,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2025-03-09</t>
+          <t>2025-03-10</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2666,10 +2666,10 @@
         <v>6</v>
       </c>
       <c r="G49" t="n">
-        <v>9840</v>
+        <v>7840</v>
       </c>
       <c r="H49" t="n">
-        <v>10610</v>
+        <v>8610</v>
       </c>
       <c r="I49" t="n">
         <v>34.8</v>
@@ -2689,7 +2689,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2025-03-22</t>
+          <t>2025-03-23</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2712,10 +2712,10 @@
         <v>8</v>
       </c>
       <c r="G50" t="n">
-        <v>16920</v>
+        <v>12920</v>
       </c>
       <c r="H50" t="n">
-        <v>15620</v>
+        <v>11620</v>
       </c>
       <c r="I50" t="n">
         <v>34.2</v>
@@ -2735,7 +2735,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2025-03-22</t>
+          <t>2025-03-23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2758,10 +2758,10 @@
         <v>8</v>
       </c>
       <c r="G51" t="n">
-        <v>19650</v>
+        <v>15650</v>
       </c>
       <c r="H51" t="n">
-        <v>20260</v>
+        <v>16260</v>
       </c>
       <c r="I51" t="n">
         <v>28.9</v>
@@ -2781,7 +2781,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2025-04-01</t>
+          <t>2025-04-02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2827,7 +2827,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>2025-04-03</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2873,7 +2873,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2025-04-04</t>
+          <t>2025-04-05</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2919,7 +2919,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2025-04-12</t>
+          <t>2025-04-13</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2942,10 +2942,10 @@
         <v>4</v>
       </c>
       <c r="G55" t="n">
-        <v>11800</v>
+        <v>9430</v>
       </c>
       <c r="H55" t="n">
-        <v>11270</v>
+        <v>8900</v>
       </c>
       <c r="I55" t="n">
         <v>32.8</v>
@@ -2965,7 +2965,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2025-04-13</t>
+          <t>2025-04-14</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3011,7 +3011,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2025-04-30</t>
+          <t>2025-05-01</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3034,10 +3034,10 @@
         <v>16</v>
       </c>
       <c r="G57" t="n">
-        <v>12900</v>
+        <v>16100</v>
       </c>
       <c r="H57" t="n">
-        <v>13010</v>
+        <v>16210</v>
       </c>
       <c r="I57" t="n">
         <v>34.2</v>
@@ -3057,7 +3057,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2025-05-01</t>
+          <t>2025-05-02</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3103,7 +3103,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2025-05-01</t>
+          <t>2025-05-02</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3149,7 +3149,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2025-05-04</t>
+          <t>2025-05-05</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3195,7 +3195,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>2025-05-08</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3241,7 +3241,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2025-05-19</t>
+          <t>2025-05-20</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2025-05-26</t>
+          <t>2025-05-27</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3333,7 +3333,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2025-06-08</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3379,7 +3379,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2025-06-13</t>
+          <t>2025-06-14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3425,7 +3425,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2025-06-15</t>
+          <t>2025-06-16</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3448,10 +3448,10 @@
         <v>3</v>
       </c>
       <c r="G66" t="n">
-        <v>10370</v>
+        <v>8370</v>
       </c>
       <c r="H66" t="n">
-        <v>9510</v>
+        <v>7510</v>
       </c>
       <c r="I66" t="n">
         <v>28.1</v>
@@ -3471,7 +3471,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2025-06-30</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3517,7 +3517,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2025-07-07</t>
+          <t>2025-07-08</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3563,7 +3563,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2025-07-09</t>
+          <t>2025-07-10</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3609,7 +3609,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2025-07-13</t>
+          <t>2025-07-14</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3655,7 +3655,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2025-07-13</t>
+          <t>2025-07-14</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3701,7 +3701,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-07-16</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3747,7 +3747,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2025-08-05</t>
+          <t>2025-08-06</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3793,7 +3793,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2025-08-11</t>
+          <t>2025-08-12</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3839,7 +3839,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2025-08-17</t>
+          <t>2025-08-18</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3862,10 +3862,10 @@
         <v>2</v>
       </c>
       <c r="G75" t="n">
-        <v>19260</v>
+        <v>15630</v>
       </c>
       <c r="H75" t="n">
-        <v>19450</v>
+        <v>15820</v>
       </c>
       <c r="I75" t="n">
         <v>23</v>
@@ -3885,7 +3885,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2025-08-18</t>
+          <t>2025-08-19</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3931,7 +3931,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2025-08-24</t>
+          <t>2025-08-25</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3954,10 +3954,10 @@
         <v>25</v>
       </c>
       <c r="G77" t="n">
-        <v>9760</v>
+        <v>7760</v>
       </c>
       <c r="H77" t="n">
-        <v>9290</v>
+        <v>7290</v>
       </c>
       <c r="I77" t="n">
         <v>24.9</v>
@@ -3977,7 +3977,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2025-08-26</t>
+          <t>2025-08-27</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4023,7 +4023,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2025-08-26</t>
+          <t>2025-08-27</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4069,7 +4069,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2025-08-28</t>
+          <t>2025-08-29</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4115,7 +4115,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2025-08-30</t>
+          <t>2025-08-31</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4138,10 +4138,10 @@
         <v>1</v>
       </c>
       <c r="G81" t="n">
-        <v>9760</v>
+        <v>11760</v>
       </c>
       <c r="H81" t="n">
-        <v>9410</v>
+        <v>11410</v>
       </c>
       <c r="I81" t="n">
         <v>23.7</v>
@@ -4161,7 +4161,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2025-08-31</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4207,7 +4207,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2025-09-05</t>
+          <t>2025-09-06</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4230,10 +4230,10 @@
         <v>14</v>
       </c>
       <c r="G83" t="n">
-        <v>9920</v>
+        <v>12290</v>
       </c>
       <c r="H83" t="n">
-        <v>8860</v>
+        <v>11230</v>
       </c>
       <c r="I83" t="n">
         <v>18.7</v>
@@ -4253,7 +4253,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4299,7 +4299,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2025-09-14</t>
+          <t>2025-09-15</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4322,10 +4322,10 @@
         <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>10590</v>
+        <v>8590</v>
       </c>
       <c r="H85" t="n">
-        <v>11470</v>
+        <v>9470</v>
       </c>
       <c r="I85" t="n">
         <v>22.5</v>
@@ -4345,7 +4345,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2025-09-14</t>
+          <t>2025-09-15</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4368,10 +4368,10 @@
         <v>16</v>
       </c>
       <c r="G86" t="n">
-        <v>8240</v>
+        <v>6240</v>
       </c>
       <c r="H86" t="n">
-        <v>8490</v>
+        <v>6490</v>
       </c>
       <c r="I86" t="n">
         <v>23.3</v>
@@ -4391,7 +4391,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2025-09-21</t>
+          <t>2025-09-22</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4414,10 +4414,10 @@
         <v>28</v>
       </c>
       <c r="G87" t="n">
-        <v>18040</v>
+        <v>14420</v>
       </c>
       <c r="H87" t="n">
-        <v>17930</v>
+        <v>14310</v>
       </c>
       <c r="I87" t="n">
         <v>21.9</v>
@@ -4437,7 +4437,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2025-09-26</t>
+          <t>2025-09-27</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4483,7 +4483,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2025-10-05</t>
+          <t>2025-10-06</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4529,7 +4529,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2025-10-13</t>
+          <t>2025-10-14</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4575,7 +4575,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-11-01</t>
+          <t>2025-11-02</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4598,10 +4598,10 @@
         <v>12</v>
       </c>
       <c r="G91" t="n">
-        <v>7590</v>
+        <v>9590</v>
       </c>
       <c r="H91" t="n">
-        <v>7670</v>
+        <v>9670</v>
       </c>
       <c r="I91" t="n">
         <v>21.1</v>
@@ -4621,7 +4621,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2025-11-02</t>
+          <t>2025-11-03</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2025-11-05</t>
+          <t>2025-11-06</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4713,7 +4713,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2025-11-06</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4759,7 +4759,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-11-08</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4782,10 +4782,10 @@
         <v>0</v>
       </c>
       <c r="G95" t="n">
-        <v>12030</v>
+        <v>14410</v>
       </c>
       <c r="H95" t="n">
-        <v>11920</v>
+        <v>14300</v>
       </c>
       <c r="I95" t="n">
         <v>20.5</v>
@@ -4805,7 +4805,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2025-11-08</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4828,10 +4828,10 @@
         <v>3</v>
       </c>
       <c r="G96" t="n">
-        <v>11610</v>
+        <v>9230</v>
       </c>
       <c r="H96" t="n">
-        <v>12280</v>
+        <v>9900</v>
       </c>
       <c r="I96" t="n">
         <v>23.1</v>
@@ -4851,7 +4851,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2025-11-08</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4874,10 +4874,10 @@
         <v>6</v>
       </c>
       <c r="G97" t="n">
-        <v>11960</v>
+        <v>9590</v>
       </c>
       <c r="H97" t="n">
-        <v>11080</v>
+        <v>8710</v>
       </c>
       <c r="I97" t="n">
         <v>18.6</v>
@@ -4897,7 +4897,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-11-14</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4943,7 +4943,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2025-11-18</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4989,7 +4989,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-11-22</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5012,10 +5012,10 @@
         <v>16</v>
       </c>
       <c r="G100" t="n">
-        <v>10080</v>
+        <v>12460</v>
       </c>
       <c r="H100" t="n">
-        <v>10190</v>
+        <v>12570</v>
       </c>
       <c r="I100" t="n">
         <v>23.4</v>
@@ -5035,7 +5035,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2025-11-22</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5058,10 +5058,10 @@
         <v>6</v>
       </c>
       <c r="G101" t="n">
-        <v>14630</v>
+        <v>18250</v>
       </c>
       <c r="H101" t="n">
-        <v>15270</v>
+        <v>18890</v>
       </c>
       <c r="I101" t="n">
         <v>22.4</v>
@@ -5081,7 +5081,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5127,7 +5127,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5173,7 +5173,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5219,7 +5219,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2025-12-06</t>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5242,10 +5242,10 @@
         <v>9</v>
       </c>
       <c r="G105" t="n">
-        <v>17420</v>
+        <v>21050</v>
       </c>
       <c r="H105" t="n">
-        <v>17200</v>
+        <v>20830</v>
       </c>
       <c r="I105" t="n">
         <v>24.1</v>
@@ -5265,7 +5265,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5311,7 +5311,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5403,7 +5403,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5449,7 +5449,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5495,7 +5495,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5518,10 +5518,10 @@
         <v>17</v>
       </c>
       <c r="G111" t="n">
-        <v>11750</v>
+        <v>9750</v>
       </c>
       <c r="H111" t="n">
-        <v>11790</v>
+        <v>9790</v>
       </c>
       <c r="I111" t="n">
         <v>24.4</v>
@@ -5541,7 +5541,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2025-12-25</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5587,7 +5587,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5610,10 +5610,10 @@
         <v>0</v>
       </c>
       <c r="G113" t="n">
-        <v>10930</v>
+        <v>12930</v>
       </c>
       <c r="H113" t="n">
-        <v>11170</v>
+        <v>13170</v>
       </c>
       <c r="I113" t="n">
         <v>20.2</v>
@@ -5633,7 +5633,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5679,7 +5679,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5702,10 +5702,10 @@
         <v>11</v>
       </c>
       <c r="G115" t="n">
-        <v>8570</v>
+        <v>6570</v>
       </c>
       <c r="H115" t="n">
-        <v>8680</v>
+        <v>6680</v>
       </c>
       <c r="I115" t="n">
         <v>20.7</v>
@@ -5725,7 +5725,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5748,10 +5748,10 @@
         <v>19</v>
       </c>
       <c r="G116" t="n">
-        <v>9740</v>
+        <v>7740</v>
       </c>
       <c r="H116" t="n">
-        <v>8000</v>
+        <v>6000</v>
       </c>
       <c r="I116" t="n">
         <v>24.4</v>
@@ -5771,7 +5771,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5817,7 +5817,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5840,10 +5840,10 @@
         <v>18</v>
       </c>
       <c r="G118" t="n">
-        <v>10350</v>
+        <v>8350</v>
       </c>
       <c r="H118" t="n">
-        <v>10880</v>
+        <v>8880</v>
       </c>
       <c r="I118" t="n">
         <v>24.8</v>
@@ -5863,7 +5863,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5909,7 +5909,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -5955,7 +5955,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6001,7 +6001,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -6093,7 +6093,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -6116,10 +6116,10 @@
         <v>17</v>
       </c>
       <c r="G124" t="n">
-        <v>8830</v>
+        <v>10830</v>
       </c>
       <c r="H124" t="n">
-        <v>8770</v>
+        <v>10770</v>
       </c>
       <c r="I124" t="n">
         <v>22.2</v>
@@ -6139,7 +6139,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -6162,30 +6162,30 @@
         <v>11</v>
       </c>
       <c r="G125" t="n">
-        <v>8820</v>
+        <v>10820</v>
       </c>
       <c r="H125" t="n">
-        <v>9400</v>
+        <v>11400</v>
       </c>
       <c r="I125" t="n">
-        <v>23.7</v>
+        <v>34.7</v>
       </c>
       <c r="J125" t="n">
-        <v>9.5</v>
+        <v>19</v>
       </c>
       <c r="K125" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>Sunny</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -6208,10 +6208,10 @@
         <v>5</v>
       </c>
       <c r="G126" t="n">
-        <v>11700</v>
+        <v>9700</v>
       </c>
       <c r="H126" t="n">
-        <v>11090</v>
+        <v>9090</v>
       </c>
       <c r="I126" t="n">
         <v>34.8</v>
@@ -6231,7 +6231,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -6277,7 +6277,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -6300,10 +6300,10 @@
         <v>1</v>
       </c>
       <c r="G128" t="n">
-        <v>19260</v>
+        <v>23260</v>
       </c>
       <c r="H128" t="n">
-        <v>20070</v>
+        <v>24070</v>
       </c>
       <c r="I128" t="n">
         <v>34</v>
@@ -6323,7 +6323,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -6369,7 +6369,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -6415,7 +6415,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -6461,7 +6461,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -6507,7 +6507,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -6553,7 +6553,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -6599,7 +6599,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6645,7 +6645,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -6668,10 +6668,10 @@
         <v>1</v>
       </c>
       <c r="G136" t="n">
-        <v>12210</v>
+        <v>14590</v>
       </c>
       <c r="H136" t="n">
-        <v>13050</v>
+        <v>15430</v>
       </c>
       <c r="I136" t="n">
         <v>36.5</v>
@@ -6691,7 +6691,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -6783,7 +6783,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6829,7 +6829,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -6875,7 +6875,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6921,7 +6921,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -6944,10 +6944,10 @@
         <v>2</v>
       </c>
       <c r="G142" t="n">
-        <v>13180</v>
+        <v>10800</v>
       </c>
       <c r="H142" t="n">
-        <v>13170</v>
+        <v>10790</v>
       </c>
       <c r="I142" t="n">
         <v>25.1</v>
@@ -6967,7 +6967,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -7013,7 +7013,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -7059,7 +7059,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -7105,7 +7105,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -7151,7 +7151,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -7197,7 +7197,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -7243,7 +7243,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -7266,10 +7266,10 @@
         <v>3</v>
       </c>
       <c r="G149" t="n">
-        <v>16020</v>
+        <v>20020</v>
       </c>
       <c r="H149" t="n">
-        <v>16020</v>
+        <v>20020</v>
       </c>
       <c r="I149" t="n">
         <v>24.8</v>
@@ -7289,7 +7289,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -7312,10 +7312,10 @@
         <v>1</v>
       </c>
       <c r="G150" t="n">
-        <v>13020</v>
+        <v>10640</v>
       </c>
       <c r="H150" t="n">
-        <v>12550</v>
+        <v>10170</v>
       </c>
       <c r="I150" t="n">
         <v>24.6</v>
@@ -7335,7 +7335,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">

</xml_diff>